<commit_message>
Phase 1b: aflatoxin tightening, فلفل→spices, nuts→cereals, sector enrichment
Per Muhannad's classification review:
- Aflatoxin valid = grains/legumes, spices, sweets (removed RTE/meat/beverage);
  184 nut rows reclassified grains/legumes.
- فلفل → spices for ALL rows (1,616) + «فلفل» name-group consolidates 74 variants.
- New chemistry/scripts/sectors.py: municipality → 5-sector taxonomy with
  normalization; adds sector + sector_flag. 12,332 rows mapped, 21 true-junk.

Regenerated all chemistry parquets + synced clean/chemistry (+ xlsx).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/chemistry/reports/classification_review_2026-07-01.xlsx
+++ b/chemistry/reports/classification_review_2026-07-01.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل، البهارات والصوصات، الحبوب والبقوليات، الحلويات والشوكولاتة</t>
+          <t>البهارات والصوصات، الحبوب والبقوليات، الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الجنوب</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ private</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ private</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الشرق</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الغرب</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في المنطقة الوسطى</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الجنوب</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الشمال</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ no_municipality</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ no_municipality</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الشمال</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في الشمال</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في المنطقة الوسطى</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في المنطقة الوسطى</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ private</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في المنطقة الوسطى</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>فرع أمانة في المنطقة الوسطى</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>★ UNMAPPED</t>
+          <t>★ unmapped</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">

</xml_diff>

<commit_message>
Add CSV mirrors + RTE_contents to classification review
CSV per table (UTF-8-BOM for Arabic in Excel) at reports/classification_review_csv/.
New RTE_contents table (550 rows) for Muhannad to rule where each ready-to-eat
item goes, since RTE→0 conflicts with the nuts→grains ruling.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/chemistry/reports/classification_review_2026-07-01.xlsx
+++ b/chemistry/reports/classification_review_2026-07-01.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="section_valid_cats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="name_keyword_rules" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="name_groups" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sector_taxonomy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="municipality_to_sector" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTE_contents" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sector_taxonomy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="municipality_to_sector" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1940,78 +1941,2828 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sector</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sub_municipalities</t>
+          <t>sample_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>count</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>فرع أمانة في الشرق</t>
+          <t>food_chemistry_2025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>الروضة، الشرق</t>
+          <t>لوز امريكي ني</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>75</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>فرع أمانة في الشمال</t>
+          <t>food_chemistry_2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>فستق امريكي ني</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>46</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>فرع أمانة في الغرب</t>
+          <t>food_chemistry_2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>العريجاء، عرقة، نمار</t>
+          <t>كاجو ني</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>فرع أمانة في المنطقة الوسطى</t>
+          <t>food_chemistry_2025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>الملز، المعذر، العليا، الشميسي، البطحاء</t>
+          <t>كاجو فيتنامي ني</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>فرع أمانة في الجنوب</t>
+          <t>food_chemistry_2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>العزيزية، الحاير، الشفا، السلي، النسيم</t>
+          <t>فستق ني</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>لوز ني امريكي</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>فستق ليمون</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>لوز ني</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>كاجو فتنامي ني</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>كاجو امريكي ني</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>لوز امريكي</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>فستق ني امريكي</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>بصل ابيض White onions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>كاجو ني فتنامي</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>فستق مالح</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>فستق ليمون امريكي</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>لوز افغاني ني</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>لوز ليمون</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>كاجو فتنامي</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>فستق امريكي</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>كاجو ني امريكي</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>بصل ابيض</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>كاجو هندي ني</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>لوز ني افغاني</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>فجل ابيض Radishes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>لوز افغاني</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>فستق امريكي بالليمون</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>فول سوداني محمص</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>كاجو مالح</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>لوز مالح</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>كاجو محمص</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>فول سوداني</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ترمس حلو</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>عسل عينة خاصة</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>عسل</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>عسل طبيعي</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>عسل</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>بصل ابيض Onions</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>لوز مدخن</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>فول سوداني مملح</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>لوز يمني ني</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>لوز امريكي مالح</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>كاجو هندي</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>heavy_metals_2025</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>زيت زيتون</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>heavy_metals_2025</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>دبس</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>heavy_metals_2025</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>عسل</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>عسل بشاور رقم 1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>عسل يمني</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>عسل زهور برية</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>عسل طلح فاخر</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>عينة خاصة عسل</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>عينة خاصة دبس</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>عسل م- ك</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>عسل سدر يمني م ك</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>عسل سدر م ك</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>عسل سدر مستورد باكستاني</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>عسل سدر حضرمي</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>عسل سدر بشاور</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>عسل زهور جبلي</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>عسل سدر اماراتي</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>عسل سمره اماراتي</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>عسل طلح محلي</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>عسل حبة البركة مستورد</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>عسل شوكة يمني</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>honey_2025</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>عسل برسيم مستورد من مصر</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>food_chemistry_2024</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>بصل مجفف ابيض</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>food_chemistry_2024</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>خبز توست ابيض</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>food_chemistry_2024</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>بصل مجفف ابيض ني</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>food_chemistry_2024</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>طحين ابيض</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>عسل بشاور رقم 1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>عسل يمني</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1مكسرات يابانيه</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>مكسرات يابانيه 2</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>رقائق بطاطس تركية1</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>عسل زهور برية</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>عسل طلح فاخر</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>دبس</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>سميد خشن</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>aflatoxins_2025</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>حبة البركة</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>pesticides_2025</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>دبس</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>pesticides_2025</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>عسل</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>فطر ابيض علبه</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>فجل ابيض</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>pesticides_2024</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>بصل أبيض White onion</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>aflatoxins_2024</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>بصل مجفف ابيض ني</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>شوكلاتة دارك</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>فستق حار</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>كاجو جامبو</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>لوز بالليمون</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>فول سوداني مالح</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>كاجو بالجبنة</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>لوز محمص</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>مشمش مجفف</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>فول سوداني ني</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>عسل بشاور رقم 1</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>عسل يمني</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1مكسرات يابانيه</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>مكسرات يابانيه 2</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>رقائق بطاطس تركية1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>رقائق بطاطس تركية 2</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>كاجو محمص بدون ملح</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>الفستق مالح</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>عسل عينة خاصة</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>عسل زهور برية</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>عسل طلح فاخر</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>كاجو نبي</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>فول سوداني مصري</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>تمر القصيم</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>لوز أمريكي ني</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>لوز محمص بدون ملح</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>لوز امركي امريكي ني</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>كاجو ليمون</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>لوز محمص سادة</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>لوز امريكي (ني)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ترمس مر</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>زبيب افغاني اسود</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>لوز يمني</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>فستق امركي ني</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>كاجو مجهول المصدر</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>فستق ليمون مجهول المصدر</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>لوز ليمون مجهول المصدر</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>كاجو محمص سادة</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>كاجو فتنامي كبير ني</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>لوز افغاني صغير</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>فستق امريكي ليمون</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>كاجو ني فيتنامي</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>كاجو فيتنامي محمص</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>لوز برازيلي</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>كاجو مشوي هندي</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>لوز خام امريكي</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>صنوبر</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>كاجو خام</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>فستق محمص امريكي</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>كاجو محمص امريكي</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>بيكان امريكي</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>كاجو وسابي</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>كاجو باربكيو</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>فستق تركي</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>بيكان</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>لوز أفغاني ني</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>فستق أمريكي ني</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>كاجو</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>كاجو اردني ني</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>شعير هندي محمص</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>كاجو ني فتناني</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>لوز مشوي</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>هيل امريكي رقم ١</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>لوز برازيلي جامبو</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>كاجو خام فيتنامي ني</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>جوز برازيلي</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>زبيب رازقي</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>لوز حلبي ني</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>لوز امريكي مدخن</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>مكسرات ياباني</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>كاجو امريكي مدخن</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>فستق ملح وليمون</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>زبيب اصفر امريكي جامو</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>لوز ليمون امريكي</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>فتسق امريكي ني</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>اللوز فتنامي</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>فستق سوري ني</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>فستق تمريكي ني</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>فستق ليمون ني</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>فستق الليمون</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>food_chemistry_2025</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>كاجو مدخن</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2026,6 +4777,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>sub_municipalities</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>فرع أمانة في الشرق</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>الروضة، الشرق</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>فرع أمانة في الشمال</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>الشمال</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>فرع أمانة في الغرب</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>العريجاء، عرقة، نمار</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>فرع أمانة في المنطقة الوسطى</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>الملز، المعذر، العليا، الشميسي، البطحاء</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>فرع أمانة في الجنوب</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>العزيزية، الحاير، الشفا، السلي، النسيم</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>